<commit_message>
Add safe Markdown migration for legacy content 6.
</commit_message>
<xml_diff>
--- a/translations/PAS_TinyMCE_Translations_EN_FA.xlsx
+++ b/translations/PAS_TinyMCE_Translations_EN_FA.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translations" sheetId="1" r:id="R4ca7d2cca7c44471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translations" sheetId="1" r:id="Rb474e3f7d41a4dfe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -78,7 +78,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -127,6 +127,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -136,7 +142,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TinyMCETranslations" displayName="TinyMCETranslations" ref="A1:B83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TinyMCETranslations" displayName="TinyMCETranslations" ref="A1:B126" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="EN"/>
     <x:tableColumn id="2" name="FA"/>
@@ -1011,10 +1017,354 @@
         <x:v>پیش‌فرض</x:v>
       </x:c>
     </x:row>
+    <x:row r="84" ht="15" hidden="0" customHeight="1">
+      <x:c r="A84" s="20" t="str">
+        <x:v>Markdown Content Migration</x:v>
+      </x:c>
+      <x:c r="B84" s="20" t="str">
+        <x:v>مهاجرت محتوای مارک‌داون</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A85" s="20" t="str">
+        <x:v>Preview and convert legacy AseqBase Markdown content to sanitized HTML for TinyMCE. PHP code is never stored in content.</x:v>
+      </x:c>
+      <x:c r="B85" s="20" t="str">
+        <x:v>پیش‌نمایش و تبدیل محتوای قدیمی مارک‌داون AseqBase به HTML امن برای TinyMCE. هیچ کد PHP در محتوا ذخیره نمی‌شود.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="15" hidden="0" customHeight="1">
+      <x:c r="A86" s="20" t="str">
+        <x:v>Safety notice</x:v>
+      </x:c>
+      <x:c r="B86" s="20" t="str">
+        <x:v>نکته ایمنی</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A87" s="20" t="str">
+        <x:v>Test this migration on a local database backup first. Mixed HTML and Markdown, unsupported directives, and content edited after migration are never overwritten automatically.</x:v>
+      </x:c>
+      <x:c r="B87" s="20" t="str">
+        <x:v>این مهاجرت را ابتدا روی نسخه پشتیبان دیتابیس محلی آزمایش کنید. محتوای ترکیبی HTML و مارک‌داون، دستورهای پشتیبانی‌نشده و محتوایی که پس از مهاجرت ویرایش شده باشد هرگز به‌صورت خودکار بازنویسی نمی‌شود.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="15" hidden="0" customHeight="1">
+      <x:c r="A88" s="20" t="str">
+        <x:v>Total content</x:v>
+      </x:c>
+      <x:c r="B88" s="20" t="str">
+        <x:v>کل محتوا</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="15" hidden="0" customHeight="1">
+      <x:c r="A89" s="20" t="str">
+        <x:v>Eligible</x:v>
+      </x:c>
+      <x:c r="B89" s="20" t="str">
+        <x:v>قابل مهاجرت</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="15" hidden="0" customHeight="1">
+      <x:c r="A90" s="20" t="str">
+        <x:v>Markdown</x:v>
+      </x:c>
+      <x:c r="B90" s="20" t="str">
+        <x:v>مارک‌داون</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="15" hidden="0" customHeight="1">
+      <x:c r="A91" s="20" t="str">
+        <x:v>Plain text</x:v>
+      </x:c>
+      <x:c r="B91" s="20" t="str">
+        <x:v>متن ساده</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="15" hidden="0" customHeight="1">
+      <x:c r="A92" s="20" t="str">
+        <x:v>Existing HTML</x:v>
+      </x:c>
+      <x:c r="B92" s="20" t="str">
+        <x:v>HTML موجود</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="15" hidden="0" customHeight="1">
+      <x:c r="A93" s="20" t="str">
+        <x:v>Mixed content</x:v>
+      </x:c>
+      <x:c r="B93" s="20" t="str">
+        <x:v>محتوای ترکیبی</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="15" hidden="0" customHeight="1">
+      <x:c r="A94" s="20" t="str">
+        <x:v>Unsupported content</x:v>
+      </x:c>
+      <x:c r="B94" s="20" t="str">
+        <x:v>محتوای پشتیبانی‌نشده</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="15" hidden="0" customHeight="1">
+      <x:c r="A95" s="20" t="str">
+        <x:v>Active backups</x:v>
+      </x:c>
+      <x:c r="B95" s="20" t="str">
+        <x:v>پشتیبان‌های فعال</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="15" hidden="0" customHeight="1">
+      <x:c r="A96" s="20" t="str">
+        <x:v>Edited after migration</x:v>
+      </x:c>
+      <x:c r="B96" s="20" t="str">
+        <x:v>ویرایش‌شده پس از مهاجرت</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="15" hidden="0" customHeight="1">
+      <x:c r="A97" s="20" t="str">
+        <x:v>Apply next migration batch</x:v>
+      </x:c>
+      <x:c r="B97" s="20" t="str">
+        <x:v>اجرای گروه بعدی مهاجرت</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A98" s="20" t="str">
+        <x:v>Original content and update time are saved in a dedicated backup table before each change.</x:v>
+      </x:c>
+      <x:c r="B98" s="20" t="str">
+        <x:v>پیش از هر تغییر، محتوای اصلی و زمان به‌روزرسانی در جدول پشتیبان اختصاصی ذخیره می‌شود.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="15" hidden="0" customHeight="1">
+      <x:c r="A99" s="20" t="str">
+        <x:v>Batch size</x:v>
+      </x:c>
+      <x:c r="B99" s="20" t="str">
+        <x:v>اندازه گروه</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="15" hidden="0" customHeight="1">
+      <x:c r="A100" s="20" t="str">
+        <x:v>Type MIGRATE to confirm</x:v>
+      </x:c>
+      <x:c r="B100" s="20" t="str">
+        <x:v>برای تأیید عبارت MIGRATE را وارد کنید</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="15" hidden="0" customHeight="1">
+      <x:c r="A101" s="20" t="str">
+        <x:v>Apply migration batch</x:v>
+      </x:c>
+      <x:c r="B101" s="20" t="str">
+        <x:v>اجرای گروه مهاجرت</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="15" hidden="0" customHeight="1">
+      <x:c r="A102" s="20" t="str">
+        <x:v>Rollback last migration batch</x:v>
+      </x:c>
+      <x:c r="B102" s="20" t="str">
+        <x:v>بازگردانی آخرین گروه مهاجرت</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A103" s="20" t="str">
+        <x:v>Records edited after migration are protected and will not be overwritten.</x:v>
+      </x:c>
+      <x:c r="B103" s="20" t="str">
+        <x:v>رکوردهایی که پس از مهاجرت ویرایش شده‌اند محافظت می‌شوند و بازنویسی نخواهند شد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="15" hidden="0" customHeight="1">
+      <x:c r="A104" s="20" t="str">
+        <x:v>Type ROLLBACK to confirm</x:v>
+      </x:c>
+      <x:c r="B104" s="20" t="str">
+        <x:v>برای تأیید عبارت ROLLBACK را وارد کنید</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="15" hidden="0" customHeight="1">
+      <x:c r="A105" s="20" t="str">
+        <x:v>Restore from migration backup</x:v>
+      </x:c>
+      <x:c r="B105" s="20" t="str">
+        <x:v>بازیابی از پشتیبان مهاجرت</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="15" hidden="0" customHeight="1">
+      <x:c r="A106" s="20" t="str">
+        <x:v>Dry-run samples</x:v>
+      </x:c>
+      <x:c r="B106" s="20" t="str">
+        <x:v>نمونه‌های پیش‌نمایش آزمایشی</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="15" hidden="0" customHeight="1">
+      <x:c r="A107" s="20" t="str">
+        <x:v>No eligible or exceptional content records were found.</x:v>
+      </x:c>
+      <x:c r="B107" s="20" t="str">
+        <x:v>هیچ محتوای قابل مهاجرت یا استثنایی پیدا نشد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="15" hidden="0" customHeight="1">
+      <x:c r="A108" s="20" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B108" s="20" t="str">
+        <x:v>شناسه</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="15" hidden="0" customHeight="1">
+      <x:c r="A109" s="20" t="str">
+        <x:v>Detected format</x:v>
+      </x:c>
+      <x:c r="B109" s="20" t="str">
+        <x:v>قالب تشخیص‌داده‌شده</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="15" hidden="0" customHeight="1">
+      <x:c r="A110" s="20" t="str">
+        <x:v>Original content</x:v>
+      </x:c>
+      <x:c r="B110" s="20" t="str">
+        <x:v>محتوای اصلی</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="15" hidden="0" customHeight="1">
+      <x:c r="A111" s="20" t="str">
+        <x:v>Converted preview</x:v>
+      </x:c>
+      <x:c r="B111" s="20" t="str">
+        <x:v>پیش‌نمایش تبدیل‌شده</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="15" hidden="0" customHeight="1">
+      <x:c r="A112" s="20" t="str">
+        <x:v>Skipped for manual review</x:v>
+      </x:c>
+      <x:c r="B112" s="20" t="str">
+        <x:v>برای بررسی دستی رد شد</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="15" hidden="0" customHeight="1">
+      <x:c r="A113" s="20" t="str">
+        <x:v>Mixed</x:v>
+      </x:c>
+      <x:c r="B113" s="20" t="str">
+        <x:v>ترکیبی</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="15" hidden="0" customHeight="1">
+      <x:c r="A114" s="20" t="str">
+        <x:v>Unsupported</x:v>
+      </x:c>
+      <x:c r="B114" s="20" t="str">
+        <x:v>پشتیبانی‌نشده</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A115" s="20" t="str">
+        <x:v>%d content records were migrated. Run another batch until Eligible becomes zero.</x:v>
+      </x:c>
+      <x:c r="B115" s="20" t="str">
+        <x:v>%d رکورد محتوا مهاجرت کرد. اجرای گروه‌ها را تا صفر شدن تعداد قابل مهاجرت ادامه دهید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A116" s="20" t="str">
+        <x:v>%d content records were restored. %d edited records were protected and skipped.</x:v>
+      </x:c>
+      <x:c r="B116" s="20" t="str">
+        <x:v>%d رکورد محتوا بازیابی شد. %d رکورد ویرایش‌شده محافظت و رد شد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="15" hidden="0" customHeight="1">
+      <x:c r="A117" s="20" t="str">
+        <x:v>The migration operation failed:</x:v>
+      </x:c>
+      <x:c r="B117" s="20" t="str">
+        <x:v>عملیات مهاجرت ناموفق بود:</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="15" hidden="0" customHeight="1">
+      <x:c r="A118" s="20" t="str">
+        <x:v>Type MIGRATE in the confirmation field before applying the migration.</x:v>
+      </x:c>
+      <x:c r="B118" s="20" t="str">
+        <x:v>پیش از اجرای مهاجرت عبارت MIGRATE را در فیلد تأیید وارد کنید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="15" hidden="0" customHeight="1">
+      <x:c r="A119" s="20" t="str">
+        <x:v>Type ROLLBACK in the confirmation field before restoring content.</x:v>
+      </x:c>
+      <x:c r="B119" s="20" t="str">
+        <x:v>پیش از بازیابی محتوا عبارت ROLLBACK را در فیلد تأیید وارد کنید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="15" hidden="0" customHeight="1">
+      <x:c r="A120" s="20" t="str">
+        <x:v>Empty</x:v>
+      </x:c>
+      <x:c r="B120" s="20" t="str">
+        <x:v>خالی</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="15" hidden="0" customHeight="1">
+      <x:c r="A121" s="20" t="str">
+        <x:v>HTML and Markdown are mixed in this record.</x:v>
+      </x:c>
+      <x:c r="B121" s="20" t="str">
+        <x:v>در این رکورد HTML و مارک‌داون با هم ترکیب شده‌اند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="15" hidden="0" customHeight="1">
+      <x:c r="A122" s="20" t="str">
+        <x:v>A legacy button contains an unsupported URL.</x:v>
+      </x:c>
+      <x:c r="B122" s="20" t="str">
+        <x:v>یکی از دکمه‌های قدیمی دارای آدرس پشتیبانی‌نشده است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="15" hidden="0" customHeight="1">
+      <x:c r="A123" s="20" t="str">
+        <x:v>Unsupported custom markup:</x:v>
+      </x:c>
+      <x:c r="B123" s="20" t="str">
+        <x:v>نشانه‌گذاری سفارشی پشتیبانی‌نشده:</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A124" s="20" t="str">
+        <x:v>Content changed while the migration was running. No records were committed.</x:v>
+      </x:c>
+      <x:c r="B124" s="20" t="str">
+        <x:v>هنگام اجرای مهاجرت محتوا تغییر کرد. هیچ رکوردی ثبت نشد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A125" s="20" t="str">
+        <x:v>Content changed while the rollback was running. No records were committed.</x:v>
+      </x:c>
+      <x:c r="B125" s="20" t="str">
+        <x:v>هنگام اجرای بازگردانی محتوا تغییر کرد. هیچ رکوردی ثبت نشد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="15" hidden="0" customHeight="1">
+      <x:c r="A126" s="20" t="str">
+        <x:v>The resolved database table name is invalid.</x:v>
+      </x:c>
+      <x:c r="B126" s="20" t="str">
+        <x:v>نام جدول دیتابیس معتبر نیست.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6f506aa6705485a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01a4e05b7818484b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>